<commit_message>
fix(upload): valor zerado na planilha da faixa vai para os erros
Antes: cliente que voltava numa planilha seguinte da mesma faixa, com o
cadastro sem parcelas, saía com valor "0,00" em vez do valor da planilha,
e linha com valor zero entrava na fila para cobrança.

Depois: se o valor em atraso do cadastro é zero, vale o valor da planilha.
Se mesmo assim o valor é zero, a linha não é cobrada: vira item de erro
"Valor zerado" na fila (aparece em Erros de envio) e o resumo do upload
lista o motivo.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WqJpZyQ18gc3Yg88WN8Hmb
</commit_message>
<xml_diff>
--- a/e2e/tests/dados/planilha_faixa.xlsx
+++ b/e2e/tests/dados/planilha_faixa.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F8"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -660,6 +660,38 @@
         </is>
       </c>
     </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>107</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Paulo Zanetti</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>66677788899</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>(11) 97777-0107</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>0,00</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>16/09/2026</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>